<commit_message>
just a tiny edit to the extra rows
</commit_message>
<xml_diff>
--- a/T-W.xlsx
+++ b/T-W.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B67DF5-BDEB-4784-8DB9-EC27771077A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E65058AC-4400-48CF-B4C0-F5C542C91B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4980" yWindow="5440" windowWidth="21600" windowHeight="11320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="10" r:id="rId1"/>
@@ -1998,17 +1998,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D0DC234-49B8-4977-ABFC-550ABAC96D08}">
   <dimension ref="A2:G330"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="3"/>
-    <col min="2" max="2" width="33.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="26.453125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="21.54296875" customWidth="1"/>
-    <col min="5" max="5" width="13.08984375" customWidth="1"/>
-    <col min="6" max="6" width="151.26953125" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" style="3"/>
+    <col min="2" max="2" width="33.5703125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="151.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>227</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>2</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>2</v>
       </c>
@@ -2169,7 +2169,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
@@ -2192,7 +2192,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>3</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>227</v>
       </c>
@@ -2307,7 +2307,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>4</v>
       </c>
@@ -2376,7 +2376,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
@@ -2399,7 +2399,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>5</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>5</v>
       </c>
@@ -2445,7 +2445,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>5</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>6</v>
       </c>
@@ -2491,7 +2491,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>6</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>6</v>
       </c>
@@ -2537,7 +2537,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>6</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>6</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>6</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>6</v>
       </c>
@@ -2629,7 +2629,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>7</v>
       </c>
@@ -2652,7 +2652,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>7</v>
       </c>
@@ -2675,7 +2675,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>7</v>
       </c>
@@ -2698,7 +2698,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>7</v>
       </c>
@@ -2721,7 +2721,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>7</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>7</v>
       </c>
@@ -2767,7 +2767,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>7</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>8</v>
       </c>
@@ -2813,7 +2813,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>8</v>
       </c>
@@ -2836,7 +2836,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>8</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>9</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>9</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>9</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>10</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>10</v>
       </c>
@@ -2974,7 +2974,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>10</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>10</v>
       </c>
@@ -3020,7 +3020,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>11</v>
       </c>
@@ -3043,7 +3043,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>11</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>11</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>11</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>12</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>12</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>12</v>
       </c>
@@ -3181,7 +3181,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>12</v>
       </c>
@@ -3204,7 +3204,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>13</v>
       </c>
@@ -3227,7 +3227,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>13</v>
       </c>
@@ -3250,7 +3250,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>13</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>13</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>14</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>14</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>14</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>14</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>15</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>15</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>15</v>
       </c>
@@ -3457,7 +3457,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>15</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>16</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>16</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>16</v>
       </c>
@@ -3549,7 +3549,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>17</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>17</v>
       </c>
@@ -3595,7 +3595,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>17</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>18</v>
       </c>
@@ -3641,7 +3641,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>18</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>18</v>
       </c>
@@ -3687,7 +3687,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>19</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>19</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>19</v>
       </c>
@@ -3756,7 +3756,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>20</v>
       </c>
@@ -3779,7 +3779,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>20</v>
       </c>
@@ -3802,7 +3802,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>20</v>
       </c>
@@ -3825,7 +3825,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>21</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>21</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>21</v>
       </c>
@@ -3894,7 +3894,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>22</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>22</v>
       </c>
@@ -3940,7 +3940,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>22</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>44</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>44</v>
       </c>
@@ -4009,7 +4009,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>44</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>46</v>
       </c>
@@ -4055,7 +4055,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>46</v>
       </c>
@@ -4078,7 +4078,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>46</v>
       </c>
@@ -4101,7 +4101,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>48</v>
       </c>
@@ -4124,7 +4124,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>48</v>
       </c>
@@ -4147,7 +4147,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>48</v>
       </c>
@@ -4170,7 +4170,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>50</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>50</v>
       </c>
@@ -4216,7 +4216,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>27</v>
       </c>
@@ -4233,7 +4233,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>27</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>28</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>28</v>
       </c>
@@ -4290,7 +4290,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>28</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>29</v>
       </c>
@@ -4330,7 +4330,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>29</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>29</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>30</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>30</v>
       </c>
@@ -4404,7 +4404,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>30</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>31</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>31</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>31</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>32</v>
       </c>
@@ -4501,7 +4501,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>32</v>
       </c>
@@ -4518,7 +4518,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>32</v>
       </c>
@@ -4541,7 +4541,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>33</v>
       </c>
@@ -4558,7 +4558,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>33</v>
       </c>
@@ -4575,7 +4575,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>33</v>
       </c>
@@ -4598,7 +4598,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>34</v>
       </c>
@@ -4615,7 +4615,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>34</v>
       </c>
@@ -4632,7 +4632,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>34</v>
       </c>
@@ -4655,7 +4655,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>35</v>
       </c>
@@ -4672,7 +4672,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>35</v>
       </c>
@@ -4689,7 +4689,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>35</v>
       </c>
@@ -4706,7 +4706,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
         <v>35</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
         <v>36</v>
       </c>
@@ -4746,7 +4746,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="3">
         <v>36</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
         <v>36</v>
       </c>
@@ -4786,7 +4786,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
         <v>37</v>
       </c>
@@ -4803,7 +4803,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="3">
         <v>37</v>
       </c>
@@ -4820,7 +4820,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="3">
         <v>37</v>
       </c>
@@ -4843,7 +4843,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
         <v>38</v>
       </c>
@@ -4860,7 +4860,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="3">
         <v>38</v>
       </c>
@@ -4877,7 +4877,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="3">
         <v>38</v>
       </c>
@@ -4900,7 +4900,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="3">
         <v>39</v>
       </c>
@@ -4917,7 +4917,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
         <v>39</v>
       </c>
@@ -4934,7 +4934,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="3">
         <v>39</v>
       </c>
@@ -4951,7 +4951,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="3">
         <v>39</v>
       </c>
@@ -4974,7 +4974,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="3">
         <v>40</v>
       </c>
@@ -4991,7 +4991,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="3">
         <v>40</v>
       </c>
@@ -5008,7 +5008,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="3">
         <v>40</v>
       </c>
@@ -5031,7 +5031,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="3">
         <v>41</v>
       </c>
@@ -5048,7 +5048,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="3">
         <v>41</v>
       </c>
@@ -5065,7 +5065,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="3">
         <v>41</v>
       </c>
@@ -5088,7 +5088,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="3">
         <v>42</v>
       </c>
@@ -5105,7 +5105,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="3">
         <v>42</v>
       </c>
@@ -5122,7 +5122,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="3">
         <v>42</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="3">
         <v>43</v>
       </c>
@@ -5162,7 +5162,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="3">
         <v>43</v>
       </c>
@@ -5179,7 +5179,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="3">
         <v>43</v>
       </c>
@@ -5202,7 +5202,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="3">
         <v>44</v>
       </c>
@@ -5219,7 +5219,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="3">
         <v>44</v>
       </c>
@@ -5236,7 +5236,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="3">
         <v>44</v>
       </c>
@@ -5259,7 +5259,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="3">
         <v>45</v>
       </c>
@@ -5276,7 +5276,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="3">
         <v>45</v>
       </c>
@@ -5293,7 +5293,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="3">
         <v>45</v>
       </c>
@@ -5316,7 +5316,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="3">
         <v>45</v>
       </c>
@@ -5339,7 +5339,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="3">
         <v>45</v>
       </c>
@@ -5362,7 +5362,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="3">
         <v>45</v>
       </c>
@@ -5385,7 +5385,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="3">
         <v>45</v>
       </c>
@@ -5408,7 +5408,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="3">
         <v>45</v>
       </c>
@@ -5431,7 +5431,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="3">
         <v>45</v>
       </c>
@@ -5454,7 +5454,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="3">
         <v>45</v>
       </c>
@@ -5477,7 +5477,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="3">
         <v>45</v>
       </c>
@@ -5500,7 +5500,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="3">
         <v>45</v>
       </c>
@@ -5523,7 +5523,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="3">
         <v>45</v>
       </c>
@@ -5546,7 +5546,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="3">
         <v>45</v>
       </c>
@@ -5569,7 +5569,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="3">
         <v>45</v>
       </c>
@@ -5592,7 +5592,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="3">
         <v>45</v>
       </c>
@@ -5615,7 +5615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="3">
         <v>45</v>
       </c>
@@ -5638,7 +5638,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="3">
         <v>45</v>
       </c>
@@ -5661,7 +5661,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="3">
         <v>45</v>
       </c>
@@ -5684,7 +5684,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="3">
         <v>45</v>
       </c>
@@ -5707,7 +5707,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="3">
         <v>45</v>
       </c>
@@ -5730,7 +5730,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="3">
         <v>45</v>
       </c>
@@ -5753,7 +5753,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="3">
         <v>45</v>
       </c>
@@ -5776,7 +5776,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="3">
         <v>45</v>
       </c>
@@ -5799,7 +5799,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="3">
         <v>45</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="3">
         <v>45</v>
       </c>
@@ -5845,7 +5845,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="3">
         <v>45</v>
       </c>
@@ -5868,7 +5868,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="3">
         <v>45</v>
       </c>
@@ -5891,7 +5891,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="3">
         <v>45</v>
       </c>
@@ -5914,7 +5914,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="3">
         <v>45</v>
       </c>
@@ -5937,7 +5937,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" s="3">
         <v>45</v>
       </c>
@@ -5960,7 +5960,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" s="3">
         <v>45</v>
       </c>
@@ -5983,7 +5983,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="3">
         <v>45</v>
       </c>
@@ -6006,7 +6006,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="3">
         <v>45</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="3">
         <v>45</v>
       </c>
@@ -6052,7 +6052,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="3">
         <v>45</v>
       </c>
@@ -6075,7 +6075,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="3">
         <v>45</v>
       </c>
@@ -6098,7 +6098,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="3">
         <v>45</v>
       </c>
@@ -6121,7 +6121,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="3">
         <v>45</v>
       </c>
@@ -6144,7 +6144,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" s="3">
         <v>45</v>
       </c>
@@ -6167,7 +6167,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" s="3">
         <v>45</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="3">
         <v>45</v>
       </c>
@@ -6213,7 +6213,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="3">
         <v>45</v>
       </c>
@@ -6236,7 +6236,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="3">
         <v>45</v>
       </c>
@@ -6259,7 +6259,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="3">
         <v>45</v>
       </c>
@@ -6282,7 +6282,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" s="3">
         <v>45</v>
       </c>
@@ -6305,7 +6305,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" s="3">
         <v>45</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" s="3">
         <v>45</v>
       </c>
@@ -6351,7 +6351,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" s="3">
         <v>45</v>
       </c>
@@ -6374,7 +6374,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" s="3">
         <v>45</v>
       </c>
@@ -6397,7 +6397,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" s="3">
         <v>45</v>
       </c>
@@ -6420,7 +6420,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" s="3">
         <v>45</v>
       </c>
@@ -6443,7 +6443,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="3">
         <v>45</v>
       </c>
@@ -6466,7 +6466,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="3">
         <v>45</v>
       </c>
@@ -6489,7 +6489,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="3">
         <v>45</v>
       </c>
@@ -6512,7 +6512,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="3">
         <v>45</v>
       </c>
@@ -6535,7 +6535,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" s="3">
         <v>45</v>
       </c>
@@ -6558,7 +6558,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="3">
         <v>45</v>
       </c>
@@ -6581,7 +6581,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="3">
         <v>45</v>
       </c>
@@ -6604,7 +6604,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" s="3">
         <v>45</v>
       </c>
@@ -6627,7 +6627,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" s="3">
         <v>45</v>
       </c>
@@ -6650,7 +6650,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="3">
         <v>45</v>
       </c>
@@ -6673,7 +6673,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" s="3">
         <v>45</v>
       </c>
@@ -6696,7 +6696,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="3">
         <v>45</v>
       </c>
@@ -6719,7 +6719,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="3">
         <v>45</v>
       </c>
@@ -6742,7 +6742,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="3">
         <v>45</v>
       </c>
@@ -6765,7 +6765,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="3">
         <v>45</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="3">
         <v>45</v>
       </c>
@@ -6811,7 +6811,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="3">
         <v>45</v>
       </c>
@@ -6834,7 +6834,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" s="3">
         <v>45</v>
       </c>
@@ -6857,7 +6857,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="3">
         <v>45</v>
       </c>
@@ -6880,7 +6880,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" s="3">
         <v>45</v>
       </c>
@@ -6903,7 +6903,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" s="3">
         <v>45</v>
       </c>
@@ -6926,7 +6926,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" s="3">
         <v>45</v>
       </c>
@@ -6949,7 +6949,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" s="3">
         <v>45</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" s="3">
         <v>45</v>
       </c>
@@ -6995,7 +6995,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" s="3">
         <v>45</v>
       </c>
@@ -7018,7 +7018,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230" s="3">
         <v>45</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231" s="3">
         <v>45</v>
       </c>
@@ -7064,7 +7064,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232" s="3">
         <v>45</v>
       </c>
@@ -7087,7 +7087,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" s="3">
         <v>45</v>
       </c>
@@ -7110,7 +7110,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234" s="3">
         <v>45</v>
       </c>
@@ -7133,7 +7133,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" s="3">
         <v>45</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236" s="3">
         <v>45</v>
       </c>
@@ -7179,7 +7179,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" s="3">
         <v>45</v>
       </c>
@@ -7202,7 +7202,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" s="3">
         <v>45</v>
       </c>
@@ -7225,7 +7225,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239" s="3">
         <v>45</v>
       </c>
@@ -7248,7 +7248,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240" s="3">
         <v>45</v>
       </c>
@@ -7271,7 +7271,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A241" s="3">
         <v>45</v>
       </c>
@@ -7294,7 +7294,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242" s="3">
         <v>45</v>
       </c>
@@ -7317,7 +7317,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243" s="3">
         <v>45</v>
       </c>
@@ -7340,7 +7340,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244" s="3">
         <v>45</v>
       </c>
@@ -7363,7 +7363,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A245" s="3">
         <v>45</v>
       </c>
@@ -7386,7 +7386,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A246" s="3">
         <v>45</v>
       </c>
@@ -7409,7 +7409,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247" s="3">
         <v>45</v>
       </c>
@@ -7432,7 +7432,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248" s="3">
         <v>45</v>
       </c>
@@ -7455,7 +7455,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A249" s="3">
         <v>45</v>
       </c>
@@ -7478,7 +7478,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250" s="3">
         <v>45</v>
       </c>
@@ -7501,7 +7501,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251" s="3">
         <v>45</v>
       </c>
@@ -7524,7 +7524,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A252" s="3">
         <v>45</v>
       </c>
@@ -7547,7 +7547,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253" s="3">
         <v>45</v>
       </c>
@@ -7570,7 +7570,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A254" s="3">
         <v>45</v>
       </c>
@@ -7593,7 +7593,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" s="3">
         <v>45</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A256" s="3">
         <v>45</v>
       </c>
@@ -7639,7 +7639,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A257" s="3">
         <v>45</v>
       </c>
@@ -7662,7 +7662,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A258" s="3">
         <v>45</v>
       </c>
@@ -7685,7 +7685,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A259" s="3">
         <v>45</v>
       </c>
@@ -7708,7 +7708,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A260" s="3">
         <v>45</v>
       </c>
@@ -7731,7 +7731,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A261" s="3">
         <v>45</v>
       </c>
@@ -7754,7 +7754,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A262" s="3">
         <v>45</v>
       </c>
@@ -7777,7 +7777,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A263" s="3">
         <v>45</v>
       </c>
@@ -7800,7 +7800,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A264" s="3">
         <v>45</v>
       </c>
@@ -7823,7 +7823,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A265" s="3">
         <v>45</v>
       </c>
@@ -7846,7 +7846,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A266" s="3">
         <v>45</v>
       </c>
@@ -7869,7 +7869,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A267" s="3">
         <v>45</v>
       </c>
@@ -7892,7 +7892,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A268" s="3">
         <v>45</v>
       </c>
@@ -7915,7 +7915,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A269" s="3">
         <v>45</v>
       </c>
@@ -7938,7 +7938,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A270" s="3">
         <v>45</v>
       </c>
@@ -7961,7 +7961,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A271" s="3">
         <v>45</v>
       </c>
@@ -7984,7 +7984,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A272" s="3">
         <v>45</v>
       </c>
@@ -8007,7 +8007,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A273" s="3">
         <v>45</v>
       </c>
@@ -8030,7 +8030,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A274" s="3">
         <v>45</v>
       </c>
@@ -8053,7 +8053,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A275" s="3">
         <v>45</v>
       </c>
@@ -8076,7 +8076,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A276" s="3">
         <v>45</v>
       </c>
@@ -8099,7 +8099,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A277" s="3">
         <v>45</v>
       </c>
@@ -8122,7 +8122,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A278" s="3">
         <v>45</v>
       </c>
@@ -8145,7 +8145,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A279" s="3">
         <v>45</v>
       </c>
@@ -8168,7 +8168,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A280" s="3">
         <v>45</v>
       </c>
@@ -8191,7 +8191,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A281" s="3">
         <v>45</v>
       </c>
@@ -8214,7 +8214,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A282" s="3">
         <v>45</v>
       </c>
@@ -8237,7 +8237,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A283" s="3">
         <v>45</v>
       </c>
@@ -8260,7 +8260,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A284" s="3">
         <v>45</v>
       </c>
@@ -8283,7 +8283,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A285" s="3">
         <v>45</v>
       </c>
@@ -8306,7 +8306,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A286" s="3">
         <v>45</v>
       </c>
@@ -8329,7 +8329,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A287" s="3">
         <v>45</v>
       </c>
@@ -8352,7 +8352,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A288" s="3">
         <v>45</v>
       </c>
@@ -8375,7 +8375,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A289" s="3">
         <v>45</v>
       </c>
@@ -8398,7 +8398,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A290" s="3">
         <v>45</v>
       </c>
@@ -8421,7 +8421,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A291" s="3">
         <v>45</v>
       </c>
@@ -8444,7 +8444,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A292" s="3">
         <v>45</v>
       </c>
@@ -8467,7 +8467,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A293" s="3">
         <v>45</v>
       </c>
@@ -8490,7 +8490,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A294" s="3">
         <v>45</v>
       </c>
@@ -8513,7 +8513,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A295" s="3">
         <v>45</v>
       </c>
@@ -8536,7 +8536,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A296" s="3">
         <v>45</v>
       </c>
@@ -8559,7 +8559,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A297" s="3">
         <v>45</v>
       </c>
@@ -8582,7 +8582,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A298" s="3">
         <v>45</v>
       </c>
@@ -8605,7 +8605,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A299" s="3">
         <v>45</v>
       </c>
@@ -8628,7 +8628,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A300" s="3">
         <v>45</v>
       </c>
@@ -8651,7 +8651,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A301" s="3">
         <v>45</v>
       </c>
@@ -8674,7 +8674,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A302" s="3">
         <v>45</v>
       </c>
@@ -8697,7 +8697,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A303" s="3">
         <v>45</v>
       </c>
@@ -8720,7 +8720,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A304" s="3">
         <v>45</v>
       </c>
@@ -8743,7 +8743,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A305" s="3">
         <v>45</v>
       </c>
@@ -8766,7 +8766,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A306" s="3">
         <v>45</v>
       </c>
@@ -8789,7 +8789,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A307" s="3">
         <v>45</v>
       </c>
@@ -8812,7 +8812,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A308" s="3">
         <v>45</v>
       </c>
@@ -8835,7 +8835,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A309" s="3">
         <v>45</v>
       </c>
@@ -8858,7 +8858,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="310" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A310" s="3">
         <v>45</v>
       </c>
@@ -8881,7 +8881,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="311" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A311" s="3">
         <v>45</v>
       </c>
@@ -8904,7 +8904,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="312" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A312" s="3">
         <v>45</v>
       </c>
@@ -8927,7 +8927,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A313" s="3">
         <v>45</v>
       </c>
@@ -8950,7 +8950,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A314" s="3">
         <v>45</v>
       </c>
@@ -8973,7 +8973,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="315" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A315" s="3">
         <v>45</v>
       </c>
@@ -8996,7 +8996,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="316" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A316" s="3">
         <v>45</v>
       </c>
@@ -9019,7 +9019,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="317" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A317" s="3">
         <v>45</v>
       </c>
@@ -9042,7 +9042,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="318" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A318" s="3">
         <v>45</v>
       </c>
@@ -9065,7 +9065,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="319" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A319" s="3">
         <v>45</v>
       </c>
@@ -9088,7 +9088,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A320" s="3">
         <v>45</v>
       </c>
@@ -9111,7 +9111,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="321" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A321" s="3">
         <v>45</v>
       </c>
@@ -9134,7 +9134,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="322" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A322" s="3">
         <v>45</v>
       </c>
@@ -9157,7 +9157,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="323" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A323" s="3">
         <v>45</v>
       </c>
@@ -9180,7 +9180,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="324" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A324" s="3">
         <v>45</v>
       </c>
@@ -9203,7 +9203,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="325" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A325" s="3">
         <v>45</v>
       </c>
@@ -9226,7 +9226,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="326" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A326" s="3">
         <v>45</v>
       </c>
@@ -9249,7 +9249,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="327" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A327" s="3">
         <v>45</v>
       </c>
@@ -9272,7 +9272,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="328" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A328" s="3">
         <v>45</v>
       </c>
@@ -9295,7 +9295,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="329" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A329" s="3">
         <v>45</v>
       </c>
@@ -9318,7 +9318,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="330" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A330" s="3">
         <v>45</v>
       </c>

</xml_diff>